<commit_message>
gitignore added + some changes on the code
</commit_message>
<xml_diff>
--- a/Working_Directory/Labeling_freq.xlsx
+++ b/Working_Directory/Labeling_freq.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/E9474E394378F15E/SPE_SS2025/IMES/Final Project/DefectRecognition/Working_Directory/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\OneDrive\SPE_SS2025\IMES\Final Project\DefectRecognition\Working_Directory\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{EBF915DB-FFC5-450E-AFC1-282AAEC953B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EB82A32-9E0E-45B2-B6B0-196A87E16AC4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C5AE5A-45C9-4CD3-A872-25D903BDACA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{80EBBB99-6C61-4DB5-AC39-50C915057846}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>case name</t>
   </si>
@@ -165,6 +165,42 @@
   </si>
   <si>
     <t>G9_P4_case91.mat</t>
+  </si>
+  <si>
+    <t>G3_P1_case35.mat</t>
+  </si>
+  <si>
+    <t>G3_P2_case35.mat</t>
+  </si>
+  <si>
+    <t>G3_P3_case35.mat</t>
+  </si>
+  <si>
+    <t>G3_P4_case35.mat</t>
+  </si>
+  <si>
+    <t>G4_P1_case46.mat</t>
+  </si>
+  <si>
+    <t>G4_P2_case46.mat</t>
+  </si>
+  <si>
+    <t>G4_P3_case46.mat</t>
+  </si>
+  <si>
+    <t>G4_P4_case46.mat</t>
+  </si>
+  <si>
+    <t>G9_P1_case95.mat</t>
+  </si>
+  <si>
+    <t>G9_P2_case95.mat</t>
+  </si>
+  <si>
+    <t>G9_P3_case95.mat</t>
+  </si>
+  <si>
+    <t>G9_P4_case95.mat</t>
   </si>
 </sst>
 </file>
@@ -220,10 +256,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -543,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D2238DE-9C47-471D-94E0-427FE7D4C1C4}">
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
@@ -739,266 +771,398 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="B18">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C18">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="B19">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C19">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="B20">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C20">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="B21">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C21">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B22">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="C22">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B23">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="C23">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B24">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="C24">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B25">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="C25">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="B26">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C26">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="B27">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C27">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="B28">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C28">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="B29">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C29">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="B30">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C30">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="B31">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C31">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B32">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C32">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B33">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C33">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B34">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C34">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="B35">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C35">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B36">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C36">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B37">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C37">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="B38">
         <v>45</v>
       </c>
       <c r="C38">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="B39">
         <v>45</v>
       </c>
       <c r="C39">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B40">
         <v>45</v>
       </c>
       <c r="C40">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B41">
+        <v>45</v>
+      </c>
+      <c r="C41">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B42">
+        <v>50</v>
+      </c>
+      <c r="C42">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B43">
+        <v>50</v>
+      </c>
+      <c r="C43">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B44">
+        <v>50</v>
+      </c>
+      <c r="C44">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B45">
+        <v>50</v>
+      </c>
+      <c r="C45">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B46">
+        <v>45</v>
+      </c>
+      <c r="C46">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B47">
+        <v>45</v>
+      </c>
+      <c r="C47">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B48">
+        <v>45</v>
+      </c>
+      <c r="C48">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B41">
-        <v>45</v>
-      </c>
-      <c r="C41">
-        <v>2</v>
+      <c r="B49">
+        <v>45</v>
+      </c>
+      <c r="C49">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B50">
+        <v>45</v>
+      </c>
+      <c r="C50">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B51">
+        <v>45</v>
+      </c>
+      <c r="C51">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B52">
+        <v>45</v>
+      </c>
+      <c r="C52">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B53">
+        <v>45</v>
+      </c>
+      <c r="C53">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>